<commit_message>
updated group -- group interactions, including oxyethylene group
</commit_message>
<xml_diff>
--- a/AIOMFAC_Documents/List_of_AIOMFAC_Maingroups_and_Subgroups.xlsx
+++ b/AIOMFAC_Documents/List_of_AIOMFAC_Maingroups_and_Subgroups.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andiz\Documents\Work_McGill\Models_Code\AIOMFAC-Program\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andiz\Documents\Work_McGill\Models_Code\AIOMFAC-program\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B50E1BF6-3F55-4546-968E-5F859B9CEEA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F44318E-76A5-4037-BE22-24D90ED774C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Groups" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="258">
   <si>
     <t>hydroxyl</t>
   </si>
@@ -616,9 +616,6 @@
   </si>
   <si>
     <t xml:space="preserve"> Extension based on Compernolle et al. (2009), (peroxy groups and organonitrate); limited support for interactions with ions;</t>
-  </si>
-  <si>
-    <t>a special oxyethylene group for use with Poly(ethylene glycols); currently not yet supported in AIOMFAC-web; extension by A.Zuend, 2008, 2016;</t>
   </si>
   <si>
     <t>main group ID</t>
@@ -770,6 +767,66 @@
   </si>
   <si>
     <t>CH[OH]</t>
+  </si>
+  <si>
+    <t>organosulfate</t>
+  </si>
+  <si>
+    <t>OSOOOH</t>
+  </si>
+  <si>
+    <t>(OSOOOH)</t>
+  </si>
+  <si>
+    <t>MeOS-</t>
+  </si>
+  <si>
+    <t>EtOS-</t>
+  </si>
+  <si>
+    <t>"(MeOS-)"</t>
+  </si>
+  <si>
+    <t>"(EtOS-)"</t>
+  </si>
+  <si>
+    <t>HSucc-</t>
+  </si>
+  <si>
+    <t>"(HSucc$^-$)"</t>
+  </si>
+  <si>
+    <t>"(HSucc-)"</t>
+  </si>
+  <si>
+    <t>Succ--</t>
+  </si>
+  <si>
+    <t>"(Succ--)"</t>
+  </si>
+  <si>
+    <t>"(Succ^{2-}$)"</t>
+  </si>
+  <si>
+    <t>"(MeOS$^{-}$)"</t>
+  </si>
+  <si>
+    <t>"(EtOS$^{-}$)"</t>
+  </si>
+  <si>
+    <t>IsopreneOS-</t>
+  </si>
+  <si>
+    <t>"(IsopreneOS-)"</t>
+  </si>
+  <si>
+    <t>"(IsopreneOS$^{-}$)"</t>
+  </si>
+  <si>
+    <t>Ion for Isoprene-OS-3/4</t>
+  </si>
+  <si>
+    <t>a special oxyethylene group for use with Poly(ethylene glycols) and other related oligomers; currently most interactions with ions are based on ether &lt;–&gt; ion interaction parameters via analogy approach</t>
   </si>
 </sst>
 </file>
@@ -863,7 +920,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -924,6 +981,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1174,7 +1237,7 @@
     <xf numFmtId="0" fontId="9" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -1209,10 +1272,6 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1233,7 +1292,6 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="7" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1248,14 +1306,6 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="2" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="4" xfId="4" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="4" xfId="4" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="5" xfId="4" applyBorder="1"/>
-    <xf numFmtId="1" fontId="11" fillId="10" borderId="12" xfId="4" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="6" xfId="4" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="4" xfId="4" quotePrefix="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="10" borderId="0" xfId="4"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1291,6 +1341,22 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="4" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="4" xfId="4" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="5" xfId="4" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="10" fillId="12" borderId="12" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="6" xfId="4" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="4" xfId="4" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Bad" xfId="4" builtinId="27"/>
@@ -1602,23 +1668,23 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:UA102"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <dimension ref="A1:UA107"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
-    <col min="2" max="2" width="12.54296875" customWidth="1"/>
-    <col min="3" max="3" width="16.453125" customWidth="1"/>
-    <col min="4" max="4" width="13.54296875" customWidth="1"/>
-    <col min="5" max="5" width="3.08984375" customWidth="1"/>
-    <col min="6" max="6" width="24.453125" customWidth="1"/>
-    <col min="7" max="7" width="29.6328125" customWidth="1"/>
-    <col min="8" max="8" width="150.90625" customWidth="1"/>
-    <col min="9" max="9" width="13.6328125" customWidth="1"/>
+    <col min="2" max="2" width="12.5546875" customWidth="1"/>
+    <col min="3" max="3" width="16.44140625" customWidth="1"/>
+    <col min="4" max="4" width="13.5546875" customWidth="1"/>
+    <col min="5" max="5" width="3.109375" customWidth="1"/>
+    <col min="6" max="6" width="24.44140625" customWidth="1"/>
+    <col min="7" max="7" width="29.6640625" customWidth="1"/>
+    <col min="8" max="8" width="150.88671875" customWidth="1"/>
+    <col min="9" max="9" width="13.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:547" s="17" customFormat="1" ht="24" customHeight="1">
-      <c r="A1" s="44" t="s">
-        <v>199</v>
+      <c r="A1" s="41" t="s">
+        <v>198</v>
       </c>
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
@@ -2599,7 +2665,7 @@
     </row>
     <row r="3" spans="1:547" s="16" customFormat="1">
       <c r="A3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="BN3"/>
       <c r="BO3"/>
@@ -3575,13 +3641,13 @@
       <c r="B5" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="41" t="s">
+      <c r="C5" s="38" t="s">
+        <v>195</v>
+      </c>
+      <c r="D5" s="40" t="s">
         <v>196</v>
       </c>
-      <c r="D5" s="43" t="s">
-        <v>197</v>
-      </c>
-      <c r="E5" s="42"/>
+      <c r="E5" s="39"/>
       <c r="F5" s="19" t="s">
         <v>33</v>
       </c>
@@ -3593,16 +3659,16 @@
       </c>
     </row>
     <row r="6" spans="1:547" ht="21.75" customHeight="1" thickBot="1">
-      <c r="A6" s="56" t="s">
+      <c r="A6" s="47" t="s">
         <v>192</v>
       </c>
-      <c r="B6" s="57"/>
-      <c r="C6" s="57"/>
-      <c r="D6" s="58"/>
-      <c r="E6" s="57"/>
-      <c r="F6" s="57"/>
-      <c r="G6" s="57"/>
-      <c r="H6" s="59"/>
+      <c r="B6" s="48"/>
+      <c r="C6" s="48"/>
+      <c r="D6" s="49"/>
+      <c r="E6" s="48"/>
+      <c r="F6" s="48"/>
+      <c r="G6" s="48"/>
+      <c r="H6" s="50"/>
     </row>
     <row r="7" spans="1:547">
       <c r="A7" s="9" t="s">
@@ -3611,13 +3677,13 @@
       <c r="B7" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="24">
+      <c r="C7" s="22">
         <v>1</v>
       </c>
-      <c r="D7" s="33">
+      <c r="D7" s="31">
         <v>1</v>
       </c>
-      <c r="E7" s="28"/>
+      <c r="E7" s="26"/>
       <c r="F7" s="11" t="s">
         <v>71</v>
       </c>
@@ -3629,11 +3695,11 @@
     <row r="8" spans="1:547">
       <c r="A8" s="9"/>
       <c r="B8" s="10"/>
-      <c r="C8" s="24"/>
-      <c r="D8" s="34">
+      <c r="C8" s="22"/>
+      <c r="D8" s="32">
         <v>2</v>
       </c>
-      <c r="E8" s="28"/>
+      <c r="E8" s="26"/>
       <c r="F8" s="11" t="s">
         <v>73</v>
       </c>
@@ -3645,11 +3711,11 @@
     <row r="9" spans="1:547">
       <c r="A9" s="9"/>
       <c r="B9" s="10"/>
-      <c r="C9" s="24"/>
-      <c r="D9" s="34">
+      <c r="C9" s="22"/>
+      <c r="D9" s="32">
         <v>3</v>
       </c>
-      <c r="E9" s="28"/>
+      <c r="E9" s="26"/>
       <c r="F9" s="11" t="s">
         <v>75</v>
       </c>
@@ -3661,11 +3727,11 @@
     <row r="10" spans="1:547">
       <c r="A10" s="9"/>
       <c r="B10" s="10"/>
-      <c r="C10" s="24"/>
-      <c r="D10" s="34">
+      <c r="C10" s="22"/>
+      <c r="D10" s="32">
         <v>4</v>
       </c>
-      <c r="E10" s="28"/>
+      <c r="E10" s="26"/>
       <c r="F10" s="11" t="s">
         <v>76</v>
       </c>
@@ -3681,13 +3747,13 @@
       <c r="B11" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="25">
+      <c r="C11" s="23">
         <v>2</v>
       </c>
-      <c r="D11" s="35">
+      <c r="D11" s="33">
         <v>5</v>
       </c>
-      <c r="E11" s="29"/>
+      <c r="E11" s="27"/>
       <c r="F11" s="6" t="s">
         <v>77</v>
       </c>
@@ -3699,11 +3765,11 @@
     <row r="12" spans="1:547">
       <c r="A12" s="5"/>
       <c r="B12" s="6"/>
-      <c r="C12" s="25"/>
-      <c r="D12" s="35">
+      <c r="C12" s="23"/>
+      <c r="D12" s="33">
         <v>6</v>
       </c>
-      <c r="E12" s="29"/>
+      <c r="E12" s="27"/>
       <c r="F12" s="6" t="s">
         <v>79</v>
       </c>
@@ -3715,11 +3781,11 @@
     <row r="13" spans="1:547">
       <c r="A13" s="5"/>
       <c r="B13" s="6"/>
-      <c r="C13" s="25"/>
-      <c r="D13" s="35">
+      <c r="C13" s="23"/>
+      <c r="D13" s="33">
         <v>7</v>
       </c>
-      <c r="E13" s="29"/>
+      <c r="E13" s="27"/>
       <c r="F13" s="6" t="s">
         <v>80</v>
       </c>
@@ -3731,11 +3797,11 @@
     <row r="14" spans="1:547">
       <c r="A14" s="5"/>
       <c r="B14" s="6"/>
-      <c r="C14" s="25"/>
-      <c r="D14" s="35">
+      <c r="C14" s="23"/>
+      <c r="D14" s="33">
         <v>8</v>
       </c>
-      <c r="E14" s="29"/>
+      <c r="E14" s="27"/>
       <c r="F14" s="6" t="s">
         <v>82</v>
       </c>
@@ -3747,11 +3813,11 @@
     <row r="15" spans="1:547">
       <c r="A15" s="5"/>
       <c r="B15" s="6"/>
-      <c r="C15" s="25"/>
-      <c r="D15" s="35">
+      <c r="C15" s="23"/>
+      <c r="D15" s="33">
         <v>70</v>
       </c>
-      <c r="E15" s="29"/>
+      <c r="E15" s="27"/>
       <c r="F15" s="6" t="s">
         <v>67</v>
       </c>
@@ -3767,13 +3833,13 @@
       <c r="B16" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C16" s="24">
+      <c r="C16" s="22">
         <v>3</v>
       </c>
-      <c r="D16" s="34">
+      <c r="D16" s="32">
         <v>9</v>
       </c>
-      <c r="E16" s="28"/>
+      <c r="E16" s="26"/>
       <c r="F16" s="10" t="s">
         <v>83</v>
       </c>
@@ -3785,11 +3851,11 @@
     <row r="17" spans="1:547">
       <c r="A17" s="9"/>
       <c r="B17" s="10"/>
-      <c r="C17" s="24"/>
-      <c r="D17" s="34">
+      <c r="C17" s="22"/>
+      <c r="D17" s="32">
         <v>10</v>
       </c>
-      <c r="E17" s="28"/>
+      <c r="E17" s="26"/>
       <c r="F17" s="10" t="s">
         <v>84</v>
       </c>
@@ -3805,13 +3871,13 @@
       <c r="B18" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="C18" s="26">
+      <c r="C18" s="24">
         <v>4</v>
       </c>
-      <c r="D18" s="36">
+      <c r="D18" s="34">
         <v>11</v>
       </c>
-      <c r="E18" s="30"/>
+      <c r="E18" s="28"/>
       <c r="F18" s="14" t="s">
         <v>85</v>
       </c>
@@ -4364,11 +4430,11 @@
     <row r="19" spans="1:547" s="2" customFormat="1">
       <c r="A19" s="13"/>
       <c r="B19" s="14"/>
-      <c r="C19" s="26"/>
-      <c r="D19" s="36">
+      <c r="C19" s="24"/>
+      <c r="D19" s="34">
         <v>12</v>
       </c>
-      <c r="E19" s="30"/>
+      <c r="E19" s="28"/>
       <c r="F19" s="14" t="s">
         <v>66</v>
       </c>
@@ -4919,11 +4985,11 @@
     <row r="20" spans="1:547" s="2" customFormat="1">
       <c r="A20" s="13"/>
       <c r="B20" s="14"/>
-      <c r="C20" s="26"/>
-      <c r="D20" s="36">
+      <c r="C20" s="24"/>
+      <c r="D20" s="34">
         <v>13</v>
       </c>
-      <c r="E20" s="30"/>
+      <c r="E20" s="28"/>
       <c r="F20" s="14" t="s">
         <v>88</v>
       </c>
@@ -5478,13 +5544,13 @@
       <c r="B21" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="25">
+      <c r="C21" s="23">
         <v>69</v>
       </c>
-      <c r="D21" s="35">
+      <c r="D21" s="33">
         <v>153</v>
       </c>
-      <c r="E21" s="29"/>
+      <c r="E21" s="27"/>
       <c r="F21" s="6" t="s">
         <v>65</v>
       </c>
@@ -5500,13 +5566,13 @@
       <c r="B22" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C22" s="24">
+      <c r="C22" s="22">
         <v>8</v>
       </c>
-      <c r="D22" s="34">
+      <c r="D22" s="32">
         <v>17</v>
       </c>
-      <c r="E22" s="28"/>
+      <c r="E22" s="26"/>
       <c r="F22" s="10" t="s">
         <v>64</v>
       </c>
@@ -5522,13 +5588,13 @@
       <c r="B23" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C23" s="24">
+      <c r="C23" s="22">
         <v>9</v>
       </c>
-      <c r="D23" s="34">
+      <c r="D23" s="32">
         <v>18</v>
       </c>
-      <c r="E23" s="28"/>
+      <c r="E23" s="26"/>
       <c r="F23" s="10" t="s">
         <v>89</v>
       </c>
@@ -5540,11 +5606,11 @@
     <row r="24" spans="1:547">
       <c r="A24" s="9"/>
       <c r="B24" s="10"/>
-      <c r="C24" s="24"/>
-      <c r="D24" s="34">
+      <c r="C24" s="22"/>
+      <c r="D24" s="32">
         <v>19</v>
       </c>
-      <c r="E24" s="28"/>
+      <c r="E24" s="26"/>
       <c r="F24" s="10" t="s">
         <v>91</v>
       </c>
@@ -5562,13 +5628,13 @@
       <c r="B25" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C25" s="25">
+      <c r="C25" s="23">
         <v>10</v>
       </c>
-      <c r="D25" s="35">
+      <c r="D25" s="33">
         <v>20</v>
       </c>
-      <c r="E25" s="29"/>
+      <c r="E25" s="27"/>
       <c r="F25" s="6" t="s">
         <v>93</v>
       </c>
@@ -5584,13 +5650,13 @@
       <c r="B26" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C26" s="24">
+      <c r="C26" s="22">
         <v>11</v>
       </c>
-      <c r="D26" s="34">
+      <c r="D26" s="32">
         <v>21</v>
       </c>
-      <c r="E26" s="28"/>
+      <c r="E26" s="26"/>
       <c r="F26" s="10" t="s">
         <v>94</v>
       </c>
@@ -5602,11 +5668,11 @@
     <row r="27" spans="1:547">
       <c r="A27" s="9"/>
       <c r="B27" s="10"/>
-      <c r="C27" s="24"/>
-      <c r="D27" s="34">
+      <c r="C27" s="22"/>
+      <c r="D27" s="32">
         <v>22</v>
       </c>
-      <c r="E27" s="28"/>
+      <c r="E27" s="26"/>
       <c r="F27" s="10" t="s">
         <v>96</v>
       </c>
@@ -5622,13 +5688,13 @@
       <c r="B28" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C28" s="25">
+      <c r="C28" s="23">
         <v>13</v>
       </c>
-      <c r="D28" s="35">
+      <c r="D28" s="33">
         <v>24</v>
       </c>
-      <c r="E28" s="29"/>
+      <c r="E28" s="27"/>
       <c r="F28" s="6" t="s">
         <v>98</v>
       </c>
@@ -5640,11 +5706,11 @@
     <row r="29" spans="1:547">
       <c r="A29" s="5"/>
       <c r="B29" s="6"/>
-      <c r="C29" s="25"/>
-      <c r="D29" s="35">
+      <c r="C29" s="23"/>
+      <c r="D29" s="33">
         <v>25</v>
       </c>
-      <c r="E29" s="29"/>
+      <c r="E29" s="27"/>
       <c r="F29" s="6" t="s">
         <v>100</v>
       </c>
@@ -5656,11 +5722,11 @@
     <row r="30" spans="1:547">
       <c r="A30" s="5"/>
       <c r="B30" s="6"/>
-      <c r="C30" s="25"/>
-      <c r="D30" s="35">
+      <c r="C30" s="23"/>
+      <c r="D30" s="33">
         <v>26</v>
       </c>
-      <c r="E30" s="31"/>
+      <c r="E30" s="29"/>
       <c r="F30" s="6" t="s">
         <v>102</v>
       </c>
@@ -5672,11 +5738,11 @@
     <row r="31" spans="1:547">
       <c r="A31" s="5"/>
       <c r="B31" s="6"/>
-      <c r="C31" s="25"/>
-      <c r="D31" s="35">
+      <c r="C31" s="23"/>
+      <c r="D31" s="33">
         <v>27</v>
       </c>
-      <c r="E31" s="29"/>
+      <c r="E31" s="27"/>
       <c r="F31" s="6" t="s">
         <v>103</v>
       </c>
@@ -5692,13 +5758,13 @@
       <c r="B32" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="C32" s="52" t="s">
-        <v>231</v>
-      </c>
-      <c r="D32" s="34">
+      <c r="C32" s="43" t="s">
+        <v>230</v>
+      </c>
+      <c r="D32" s="32">
         <v>137</v>
       </c>
-      <c r="E32" s="28"/>
+      <c r="E32" s="26"/>
       <c r="F32" s="10" t="s">
         <v>63</v>
       </c>
@@ -5706,17 +5772,17 @@
         <v>63</v>
       </c>
       <c r="H32" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="33" spans="1:8">
       <c r="A33" s="9"/>
       <c r="B33" s="10"/>
-      <c r="C33" s="24"/>
-      <c r="D33" s="37">
+      <c r="C33" s="22"/>
+      <c r="D33" s="35">
         <v>43</v>
       </c>
-      <c r="E33" s="28"/>
+      <c r="E33" s="26"/>
       <c r="F33" s="10" t="s">
         <v>105</v>
       </c>
@@ -5732,13 +5798,13 @@
       <c r="B34" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="C34" s="25">
+      <c r="C34" s="23">
         <v>66</v>
       </c>
-      <c r="D34" s="35">
+      <c r="D34" s="33">
         <v>141</v>
       </c>
-      <c r="E34" s="29"/>
+      <c r="E34" s="27"/>
       <c r="F34" s="7" t="s">
         <v>106</v>
       </c>
@@ -5752,11 +5818,11 @@
     <row r="35" spans="1:8">
       <c r="A35" s="5"/>
       <c r="B35" s="6"/>
-      <c r="C35" s="25"/>
-      <c r="D35" s="35">
+      <c r="C35" s="23"/>
+      <c r="D35" s="33">
         <v>142</v>
       </c>
-      <c r="E35" s="29"/>
+      <c r="E35" s="27"/>
       <c r="F35" s="7" t="s">
         <v>108</v>
       </c>
@@ -5768,11 +5834,11 @@
     <row r="36" spans="1:8">
       <c r="A36" s="5"/>
       <c r="B36" s="6"/>
-      <c r="C36" s="25"/>
-      <c r="D36" s="35">
+      <c r="C36" s="23"/>
+      <c r="D36" s="33">
         <v>143</v>
       </c>
-      <c r="E36" s="29"/>
+      <c r="E36" s="27"/>
       <c r="F36" s="7" t="s">
         <v>110</v>
       </c>
@@ -5784,11 +5850,11 @@
     <row r="37" spans="1:8">
       <c r="A37" s="5"/>
       <c r="B37" s="6"/>
-      <c r="C37" s="25"/>
-      <c r="D37" s="35">
+      <c r="C37" s="23"/>
+      <c r="D37" s="33">
         <v>144</v>
       </c>
-      <c r="E37" s="29"/>
+      <c r="E37" s="27"/>
       <c r="F37" s="7" t="s">
         <v>112</v>
       </c>
@@ -5797,20 +5863,20 @@
       </c>
       <c r="H37" s="6"/>
     </row>
-    <row r="38" spans="1:8" ht="29">
+    <row r="38" spans="1:8" ht="28.8">
       <c r="A38" s="9" t="s">
         <v>31</v>
       </c>
       <c r="B38" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="C38" s="24">
+      <c r="C38" s="22">
         <v>67</v>
       </c>
-      <c r="D38" s="34">
+      <c r="D38" s="32">
         <v>145</v>
       </c>
-      <c r="E38" s="28"/>
+      <c r="E38" s="26"/>
       <c r="F38" s="11" t="s">
         <v>114</v>
       </c>
@@ -5824,11 +5890,11 @@
     <row r="39" spans="1:8">
       <c r="A39" s="9"/>
       <c r="B39" s="10"/>
-      <c r="C39" s="24"/>
-      <c r="D39" s="34">
+      <c r="C39" s="22"/>
+      <c r="D39" s="32">
         <v>146</v>
       </c>
-      <c r="E39" s="28"/>
+      <c r="E39" s="26"/>
       <c r="F39" s="11" t="s">
         <v>116</v>
       </c>
@@ -5840,11 +5906,11 @@
     <row r="40" spans="1:8">
       <c r="A40" s="9"/>
       <c r="B40" s="10"/>
-      <c r="C40" s="24"/>
-      <c r="D40" s="34">
+      <c r="C40" s="22"/>
+      <c r="D40" s="32">
         <v>147</v>
       </c>
-      <c r="E40" s="28"/>
+      <c r="E40" s="26"/>
       <c r="F40" s="11" t="s">
         <v>118</v>
       </c>
@@ -5856,11 +5922,11 @@
     <row r="41" spans="1:8">
       <c r="A41" s="9"/>
       <c r="B41" s="10"/>
-      <c r="C41" s="24"/>
-      <c r="D41" s="34">
+      <c r="C41" s="22"/>
+      <c r="D41" s="32">
         <v>148</v>
       </c>
-      <c r="E41" s="28"/>
+      <c r="E41" s="26"/>
       <c r="F41" s="11" t="s">
         <v>120</v>
       </c>
@@ -5869,20 +5935,20 @@
       </c>
       <c r="H41" s="10"/>
     </row>
-    <row r="42" spans="1:8" ht="29">
+    <row r="42" spans="1:8" ht="28.8">
       <c r="A42" s="5" t="s">
         <v>7</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>235</v>
-      </c>
-      <c r="C42" s="25">
+        <v>234</v>
+      </c>
+      <c r="C42" s="23">
         <v>68</v>
       </c>
-      <c r="D42" s="35">
+      <c r="D42" s="33">
         <v>149</v>
       </c>
-      <c r="E42" s="29"/>
+      <c r="E42" s="27"/>
       <c r="F42" s="7" t="s">
         <v>122</v>
       </c>
@@ -5896,11 +5962,11 @@
     <row r="43" spans="1:8">
       <c r="A43" s="5"/>
       <c r="B43" s="6"/>
-      <c r="C43" s="25"/>
-      <c r="D43" s="35">
+      <c r="C43" s="23"/>
+      <c r="D43" s="33">
         <v>150</v>
       </c>
-      <c r="E43" s="29"/>
+      <c r="E43" s="27"/>
       <c r="F43" s="7" t="s">
         <v>124</v>
       </c>
@@ -5908,15 +5974,15 @@
         <v>125</v>
       </c>
       <c r="H43" s="6" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="44" spans="1:8">
       <c r="A44" s="5"/>
       <c r="B44" s="6"/>
-      <c r="C44" s="25"/>
-      <c r="D44" s="35"/>
-      <c r="E44" s="29"/>
+      <c r="C44" s="23"/>
+      <c r="D44" s="33"/>
+      <c r="E44" s="27"/>
       <c r="F44" s="7"/>
       <c r="G44" s="7"/>
       <c r="H44" s="6"/>
@@ -5924,15 +5990,15 @@
     <row r="45" spans="1:8">
       <c r="A45" s="5"/>
       <c r="B45" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="C45" s="55">
+        <v>237</v>
+      </c>
+      <c r="C45" s="46">
         <v>52</v>
       </c>
-      <c r="D45" s="35">
+      <c r="D45" s="33">
         <v>151</v>
       </c>
-      <c r="E45" s="29"/>
+      <c r="E45" s="27"/>
       <c r="F45" s="7" t="s">
         <v>126</v>
       </c>
@@ -5940,17 +6006,17 @@
         <v>127</v>
       </c>
       <c r="H45" s="6" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="46" spans="1:8">
       <c r="A46" s="8"/>
       <c r="B46" s="6"/>
-      <c r="C46" s="25"/>
-      <c r="D46" s="35">
+      <c r="C46" s="23"/>
+      <c r="D46" s="33">
         <v>152</v>
       </c>
-      <c r="E46" s="29"/>
+      <c r="E46" s="27"/>
       <c r="F46" s="7" t="s">
         <v>128</v>
       </c>
@@ -5962,43 +6028,43 @@
     <row r="47" spans="1:8">
       <c r="A47" s="8"/>
       <c r="B47" s="6"/>
-      <c r="C47" s="25"/>
-      <c r="D47" s="35"/>
-      <c r="E47" s="29"/>
+      <c r="C47" s="23"/>
+      <c r="D47" s="33"/>
+      <c r="E47" s="27"/>
       <c r="F47" s="6"/>
       <c r="G47" s="7"/>
       <c r="H47" s="6"/>
     </row>
     <row r="48" spans="1:8">
-      <c r="A48" s="20" t="s">
+      <c r="A48" s="55" t="s">
         <v>132</v>
       </c>
-      <c r="B48" s="14" t="s">
+      <c r="B48" s="56" t="s">
         <v>133</v>
       </c>
-      <c r="C48" s="26">
+      <c r="C48" s="57">
         <v>70</v>
       </c>
-      <c r="D48" s="38">
+      <c r="D48" s="58">
         <v>154</v>
       </c>
-      <c r="E48" s="30"/>
-      <c r="F48" s="21" t="s">
+      <c r="E48" s="59"/>
+      <c r="F48" s="60" t="s">
         <v>130</v>
       </c>
-      <c r="G48" s="21" t="s">
+      <c r="G48" s="60" t="s">
         <v>131</v>
       </c>
-      <c r="H48" s="14" t="s">
-        <v>195</v>
+      <c r="H48" s="56" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="49" spans="1:8">
       <c r="A49" s="8"/>
       <c r="B49" s="6"/>
-      <c r="C49" s="25"/>
-      <c r="D49" s="35"/>
-      <c r="E49" s="29"/>
+      <c r="C49" s="23"/>
+      <c r="D49" s="33"/>
+      <c r="E49" s="27"/>
       <c r="F49" s="7"/>
       <c r="G49" s="7"/>
       <c r="H49" s="6"/>
@@ -6010,13 +6076,13 @@
       <c r="B50" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="C50" s="24">
+      <c r="C50" s="22">
         <v>71</v>
       </c>
-      <c r="D50" s="34">
+      <c r="D50" s="32">
         <v>155</v>
       </c>
-      <c r="E50" s="28"/>
+      <c r="E50" s="26"/>
       <c r="F50" s="11" t="s">
         <v>144</v>
       </c>
@@ -6030,11 +6096,11 @@
     <row r="51" spans="1:8">
       <c r="A51" s="12"/>
       <c r="B51" s="10"/>
-      <c r="C51" s="24"/>
-      <c r="D51" s="34">
+      <c r="C51" s="22"/>
+      <c r="D51" s="32">
         <v>156</v>
       </c>
-      <c r="E51" s="28"/>
+      <c r="E51" s="26"/>
       <c r="F51" s="11" t="s">
         <v>148</v>
       </c>
@@ -6046,11 +6112,11 @@
     <row r="52" spans="1:8">
       <c r="A52" s="12"/>
       <c r="B52" s="10"/>
-      <c r="C52" s="24"/>
-      <c r="D52" s="34">
+      <c r="C52" s="22"/>
+      <c r="D52" s="32">
         <v>157</v>
       </c>
-      <c r="E52" s="28"/>
+      <c r="E52" s="26"/>
       <c r="F52" s="11" t="s">
         <v>150</v>
       </c>
@@ -6066,13 +6132,13 @@
       <c r="B53" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="C53" s="25">
+      <c r="C53" s="23">
         <v>72</v>
       </c>
-      <c r="D53" s="35">
+      <c r="D53" s="33">
         <v>158</v>
       </c>
-      <c r="E53" s="29"/>
+      <c r="E53" s="27"/>
       <c r="F53" s="7" t="s">
         <v>152</v>
       </c>
@@ -6086,11 +6152,11 @@
     <row r="54" spans="1:8">
       <c r="A54" s="8"/>
       <c r="B54" s="6"/>
-      <c r="C54" s="25"/>
-      <c r="D54" s="35">
+      <c r="C54" s="23"/>
+      <c r="D54" s="33">
         <v>159</v>
       </c>
-      <c r="E54" s="29"/>
+      <c r="E54" s="27"/>
       <c r="F54" s="7" t="s">
         <v>154</v>
       </c>
@@ -6102,11 +6168,11 @@
     <row r="55" spans="1:8">
       <c r="A55" s="8"/>
       <c r="B55" s="6"/>
-      <c r="C55" s="25"/>
-      <c r="D55" s="35">
+      <c r="C55" s="23"/>
+      <c r="D55" s="33">
         <v>160</v>
       </c>
-      <c r="E55" s="29"/>
+      <c r="E55" s="27"/>
       <c r="F55" s="7" t="s">
         <v>156</v>
       </c>
@@ -6122,13 +6188,13 @@
       <c r="B56" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="C56" s="24">
+      <c r="C56" s="22">
         <v>73</v>
       </c>
-      <c r="D56" s="34">
+      <c r="D56" s="32">
         <v>161</v>
       </c>
-      <c r="E56" s="28"/>
+      <c r="E56" s="26"/>
       <c r="F56" s="11" t="s">
         <v>158</v>
       </c>
@@ -6140,23 +6206,23 @@
       </c>
     </row>
     <row r="57" spans="1:8">
-      <c r="A57" s="22" t="s">
+      <c r="A57" s="20" t="s">
         <v>140</v>
       </c>
       <c r="B57" s="15" t="s">
         <v>141</v>
       </c>
-      <c r="C57" s="27">
+      <c r="C57" s="25">
         <v>74</v>
       </c>
-      <c r="D57" s="39">
+      <c r="D57" s="36">
         <v>162</v>
       </c>
-      <c r="E57" s="32"/>
-      <c r="F57" s="23" t="s">
+      <c r="E57" s="30"/>
+      <c r="F57" s="21" t="s">
         <v>160</v>
       </c>
-      <c r="G57" s="23" t="s">
+      <c r="G57" s="21" t="s">
         <v>161</v>
       </c>
       <c r="H57" s="15" t="s">
@@ -6164,145 +6230,145 @@
       </c>
     </row>
     <row r="58" spans="1:8">
-      <c r="A58" s="22"/>
+      <c r="A58" s="20"/>
       <c r="B58" s="15"/>
-      <c r="C58" s="27"/>
-      <c r="D58" s="39">
+      <c r="C58" s="25"/>
+      <c r="D58" s="36">
         <v>163</v>
       </c>
-      <c r="E58" s="32"/>
-      <c r="F58" s="23" t="s">
+      <c r="E58" s="30"/>
+      <c r="F58" s="21" t="s">
         <v>162</v>
       </c>
-      <c r="G58" s="23" t="s">
+      <c r="G58" s="21" t="s">
         <v>163</v>
       </c>
       <c r="H58" s="15"/>
     </row>
     <row r="59" spans="1:8">
-      <c r="A59" s="22"/>
+      <c r="A59" s="20"/>
       <c r="B59" s="15"/>
-      <c r="C59" s="27"/>
-      <c r="D59" s="39">
+      <c r="C59" s="25"/>
+      <c r="D59" s="36">
         <v>164</v>
       </c>
-      <c r="E59" s="32"/>
-      <c r="F59" s="23" t="s">
+      <c r="E59" s="30"/>
+      <c r="F59" s="21" t="s">
         <v>164</v>
       </c>
-      <c r="G59" s="23" t="s">
+      <c r="G59" s="21" t="s">
         <v>165</v>
       </c>
       <c r="H59" s="15"/>
     </row>
     <row r="60" spans="1:8">
-      <c r="A60" s="22"/>
+      <c r="A60" s="20"/>
       <c r="B60" s="15"/>
-      <c r="C60" s="27"/>
-      <c r="D60" s="39">
+      <c r="C60" s="25"/>
+      <c r="D60" s="36">
         <v>165</v>
       </c>
-      <c r="E60" s="32"/>
-      <c r="F60" s="23" t="s">
+      <c r="E60" s="30"/>
+      <c r="F60" s="21" t="s">
         <v>166</v>
       </c>
-      <c r="G60" s="23" t="s">
+      <c r="G60" s="21" t="s">
         <v>167</v>
       </c>
       <c r="H60" s="15"/>
     </row>
     <row r="61" spans="1:8">
-      <c r="A61" s="22"/>
+      <c r="A61" s="20"/>
       <c r="B61" s="15"/>
-      <c r="C61" s="27"/>
-      <c r="D61" s="39">
+      <c r="C61" s="25"/>
+      <c r="D61" s="36">
         <v>166</v>
       </c>
-      <c r="E61" s="32"/>
-      <c r="F61" s="23" t="s">
+      <c r="E61" s="30"/>
+      <c r="F61" s="21" t="s">
         <v>168</v>
       </c>
-      <c r="G61" s="23" t="s">
+      <c r="G61" s="21" t="s">
         <v>169</v>
       </c>
       <c r="H61" s="15"/>
     </row>
     <row r="62" spans="1:8">
-      <c r="A62" s="22"/>
+      <c r="A62" s="20"/>
       <c r="B62" s="15"/>
-      <c r="C62" s="27"/>
-      <c r="D62" s="39">
+      <c r="C62" s="25"/>
+      <c r="D62" s="36">
         <v>167</v>
       </c>
-      <c r="E62" s="32"/>
-      <c r="F62" s="23" t="s">
+      <c r="E62" s="30"/>
+      <c r="F62" s="21" t="s">
         <v>170</v>
       </c>
-      <c r="G62" s="23" t="s">
+      <c r="G62" s="21" t="s">
         <v>171</v>
       </c>
       <c r="H62" s="15"/>
     </row>
     <row r="63" spans="1:8">
-      <c r="A63" s="22"/>
+      <c r="A63" s="20"/>
       <c r="B63" s="15"/>
-      <c r="C63" s="27"/>
-      <c r="D63" s="39">
+      <c r="C63" s="25"/>
+      <c r="D63" s="36">
         <v>168</v>
       </c>
-      <c r="E63" s="32"/>
-      <c r="F63" s="23" t="s">
+      <c r="E63" s="30"/>
+      <c r="F63" s="21" t="s">
         <v>172</v>
       </c>
-      <c r="G63" s="23" t="s">
+      <c r="G63" s="21" t="s">
         <v>173</v>
       </c>
       <c r="H63" s="15"/>
     </row>
     <row r="64" spans="1:8">
-      <c r="A64" s="22"/>
+      <c r="A64" s="20"/>
       <c r="B64" s="15"/>
-      <c r="C64" s="27"/>
-      <c r="D64" s="39">
+      <c r="C64" s="25"/>
+      <c r="D64" s="36">
         <v>169</v>
       </c>
-      <c r="E64" s="32"/>
-      <c r="F64" s="23" t="s">
+      <c r="E64" s="30"/>
+      <c r="F64" s="21" t="s">
         <v>174</v>
       </c>
-      <c r="G64" s="23" t="s">
+      <c r="G64" s="21" t="s">
         <v>175</v>
       </c>
       <c r="H64" s="15"/>
     </row>
     <row r="65" spans="1:547">
-      <c r="A65" s="22"/>
+      <c r="A65" s="20"/>
       <c r="B65" s="15"/>
-      <c r="C65" s="27"/>
-      <c r="D65" s="39">
+      <c r="C65" s="25"/>
+      <c r="D65" s="36">
         <v>170</v>
       </c>
-      <c r="E65" s="32"/>
-      <c r="F65" s="23" t="s">
+      <c r="E65" s="30"/>
+      <c r="F65" s="21" t="s">
         <v>176</v>
       </c>
-      <c r="G65" s="23" t="s">
+      <c r="G65" s="21" t="s">
         <v>177</v>
       </c>
       <c r="H65" s="15"/>
     </row>
     <row r="66" spans="1:547">
-      <c r="A66" s="22"/>
+      <c r="A66" s="20"/>
       <c r="B66" s="15"/>
-      <c r="C66" s="27"/>
-      <c r="D66" s="39">
+      <c r="C66" s="25"/>
+      <c r="D66" s="36">
         <v>171</v>
       </c>
-      <c r="E66" s="32"/>
-      <c r="F66" s="23" t="s">
+      <c r="E66" s="30"/>
+      <c r="F66" s="21" t="s">
         <v>178</v>
       </c>
-      <c r="G66" s="23" t="s">
+      <c r="G66" s="21" t="s">
         <v>179</v>
       </c>
       <c r="H66" s="15"/>
@@ -6314,13 +6380,13 @@
       <c r="B67" s="10" t="s">
         <v>143</v>
       </c>
-      <c r="C67" s="24">
+      <c r="C67" s="22">
         <v>75</v>
       </c>
-      <c r="D67" s="34">
+      <c r="D67" s="32">
         <v>172</v>
       </c>
-      <c r="E67" s="28"/>
+      <c r="E67" s="26"/>
       <c r="F67" s="11" t="s">
         <v>147</v>
       </c>
@@ -6331,59 +6397,71 @@
         <v>194</v>
       </c>
     </row>
-    <row r="68" spans="1:547" s="51" customFormat="1">
-      <c r="A68" s="45" t="s">
+    <row r="68" spans="1:547" s="42" customFormat="1">
+      <c r="A68" s="61" t="s">
+        <v>211</v>
+      </c>
+      <c r="B68" s="62" t="s">
         <v>212</v>
       </c>
-      <c r="B68" s="46" t="s">
+      <c r="C68" s="63">
+        <v>76</v>
+      </c>
+      <c r="D68" s="64">
+        <v>173</v>
+      </c>
+      <c r="E68" s="65"/>
+      <c r="F68" s="66" t="s">
         <v>213</v>
       </c>
-      <c r="C68" s="47">
-        <v>76</v>
-      </c>
-      <c r="D68" s="48">
-        <v>173</v>
-      </c>
-      <c r="E68" s="49"/>
-      <c r="F68" s="50" t="s">
+      <c r="G68" s="66" t="s">
         <v>214</v>
       </c>
-      <c r="G68" s="50" t="s">
-        <v>215</v>
-      </c>
-      <c r="H68" s="46" t="s">
-        <v>234</v>
+      <c r="H68" s="62" t="s">
+        <v>233</v>
       </c>
     </row>
     <row r="69" spans="1:547">
-      <c r="A69" s="8"/>
-      <c r="B69" s="6"/>
-      <c r="C69" s="25"/>
-      <c r="D69" s="35"/>
-      <c r="E69" s="29"/>
-      <c r="F69" s="7"/>
-      <c r="G69" s="7"/>
+      <c r="A69" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="B69" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="C69" s="23">
+        <v>53</v>
+      </c>
+      <c r="D69" s="33">
+        <v>174</v>
+      </c>
+      <c r="E69" s="27"/>
+      <c r="F69" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="G69" s="7" t="s">
+        <v>240</v>
+      </c>
       <c r="H69" s="6"/>
     </row>
     <row r="70" spans="1:547">
       <c r="A70" s="8"/>
       <c r="B70" s="6"/>
-      <c r="C70" s="25"/>
-      <c r="D70" s="35"/>
-      <c r="E70" s="29"/>
+      <c r="C70" s="23"/>
+      <c r="D70" s="33"/>
+      <c r="E70" s="27"/>
       <c r="F70" s="7"/>
       <c r="G70" s="7"/>
       <c r="H70" s="6"/>
     </row>
     <row r="71" spans="1:547" s="3" customFormat="1" ht="15" thickBot="1">
-      <c r="A71" s="63"/>
-      <c r="B71" s="63"/>
-      <c r="C71" s="63"/>
-      <c r="D71" s="63"/>
-      <c r="E71" s="63"/>
-      <c r="F71" s="63"/>
-      <c r="G71" s="63"/>
-      <c r="H71" s="63"/>
+      <c r="A71" s="54"/>
+      <c r="B71" s="54"/>
+      <c r="C71" s="54"/>
+      <c r="D71" s="54"/>
+      <c r="E71" s="54"/>
+      <c r="F71" s="54"/>
+      <c r="G71" s="54"/>
+      <c r="H71" s="54"/>
       <c r="I71"/>
       <c r="J71"/>
       <c r="K71"/>
@@ -6924,28 +7002,28 @@
       <c r="TZ71"/>
       <c r="UA71"/>
     </row>
-    <row r="72" spans="1:547" ht="19" thickTop="1">
-      <c r="A72" s="60" t="s">
+    <row r="72" spans="1:547" ht="18.600000000000001" thickTop="1">
+      <c r="A72" s="51" t="s">
         <v>191</v>
       </c>
-      <c r="B72" s="61"/>
-      <c r="C72" s="61"/>
-      <c r="D72" s="61"/>
-      <c r="E72" s="61"/>
-      <c r="F72" s="61"/>
-      <c r="G72" s="61"/>
-      <c r="H72" s="62"/>
+      <c r="B72" s="52"/>
+      <c r="C72" s="52"/>
+      <c r="D72" s="52"/>
+      <c r="E72" s="52"/>
+      <c r="F72" s="52"/>
+      <c r="G72" s="52"/>
+      <c r="H72" s="53"/>
     </row>
     <row r="73" spans="1:547">
       <c r="A73" s="8" t="s">
         <v>20</v>
       </c>
       <c r="B73" s="6"/>
-      <c r="C73" s="25"/>
-      <c r="D73" s="40">
+      <c r="C73" s="23"/>
+      <c r="D73" s="37">
         <v>205</v>
       </c>
-      <c r="E73" s="29"/>
+      <c r="E73" s="27"/>
       <c r="F73" s="6" t="s">
         <v>36</v>
       </c>
@@ -6959,11 +7037,11 @@
         <v>21</v>
       </c>
       <c r="B74" s="6"/>
-      <c r="C74" s="25"/>
-      <c r="D74" s="40">
+      <c r="C74" s="23"/>
+      <c r="D74" s="37">
         <v>201</v>
       </c>
-      <c r="E74" s="29"/>
+      <c r="E74" s="27"/>
       <c r="F74" s="6" t="s">
         <v>37</v>
       </c>
@@ -6977,11 +7055,11 @@
         <v>186</v>
       </c>
       <c r="B75" s="6"/>
-      <c r="C75" s="25"/>
-      <c r="D75" s="40">
+      <c r="C75" s="23"/>
+      <c r="D75" s="37">
         <v>202</v>
       </c>
-      <c r="E75" s="29"/>
+      <c r="E75" s="27"/>
       <c r="F75" s="6" t="s">
         <v>49</v>
       </c>
@@ -6995,11 +7073,11 @@
         <v>22</v>
       </c>
       <c r="B76" s="6"/>
-      <c r="C76" s="25"/>
-      <c r="D76" s="40">
+      <c r="C76" s="23"/>
+      <c r="D76" s="37">
         <v>203</v>
       </c>
-      <c r="E76" s="29"/>
+      <c r="E76" s="27"/>
       <c r="F76" s="6" t="s">
         <v>38</v>
       </c>
@@ -7013,11 +7091,11 @@
         <v>23</v>
       </c>
       <c r="B77" s="6"/>
-      <c r="C77" s="25"/>
-      <c r="D77" s="40">
+      <c r="C77" s="23"/>
+      <c r="D77" s="37">
         <v>204</v>
       </c>
-      <c r="E77" s="29"/>
+      <c r="E77" s="27"/>
       <c r="F77" s="6" t="s">
         <v>39</v>
       </c>
@@ -7031,11 +7109,11 @@
         <v>188</v>
       </c>
       <c r="B78" s="6"/>
-      <c r="C78" s="25"/>
-      <c r="D78" s="40">
+      <c r="C78" s="23"/>
+      <c r="D78" s="37">
         <v>223</v>
       </c>
-      <c r="E78" s="29"/>
+      <c r="E78" s="27"/>
       <c r="F78" s="6" t="s">
         <v>40</v>
       </c>
@@ -7049,11 +7127,11 @@
         <v>189</v>
       </c>
       <c r="B79" s="6"/>
-      <c r="C79" s="25"/>
-      <c r="D79" s="40">
+      <c r="C79" s="23"/>
+      <c r="D79" s="37">
         <v>221</v>
       </c>
-      <c r="E79" s="29"/>
+      <c r="E79" s="27"/>
       <c r="F79" s="6" t="s">
         <v>41</v>
       </c>
@@ -7067,11 +7145,11 @@
         <v>24</v>
       </c>
       <c r="B80" s="6"/>
-      <c r="C80" s="25"/>
-      <c r="D80" s="40">
+      <c r="C80" s="23"/>
+      <c r="D80" s="37">
         <v>242</v>
       </c>
-      <c r="E80" s="29"/>
+      <c r="E80" s="27"/>
       <c r="F80" s="6" t="s">
         <v>42</v>
       </c>
@@ -7085,11 +7163,11 @@
         <v>25</v>
       </c>
       <c r="B81" s="6"/>
-      <c r="C81" s="25"/>
-      <c r="D81" s="40">
+      <c r="C81" s="23"/>
+      <c r="D81" s="37">
         <v>243</v>
       </c>
-      <c r="E81" s="29"/>
+      <c r="E81" s="27"/>
       <c r="F81" s="6" t="s">
         <v>43</v>
       </c>
@@ -7100,19 +7178,19 @@
     </row>
     <row r="82" spans="1:8">
       <c r="A82" s="8" t="s">
+        <v>199</v>
+      </c>
+      <c r="B82" s="6"/>
+      <c r="C82" s="23"/>
+      <c r="D82" s="37">
+        <v>244</v>
+      </c>
+      <c r="E82" s="27"/>
+      <c r="F82" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="B82" s="6"/>
-      <c r="C82" s="25"/>
-      <c r="D82" s="40">
-        <v>244</v>
-      </c>
-      <c r="E82" s="29"/>
-      <c r="F82" s="6" t="s">
+      <c r="G82" s="6" t="s">
         <v>201</v>
-      </c>
-      <c r="G82" s="6" t="s">
-        <v>202</v>
       </c>
       <c r="H82" s="6"/>
     </row>
@@ -7121,11 +7199,11 @@
         <v>26</v>
       </c>
       <c r="B83" s="6"/>
-      <c r="C83" s="25"/>
-      <c r="D83" s="40">
+      <c r="C83" s="23"/>
+      <c r="D83" s="37">
         <v>245</v>
       </c>
-      <c r="E83" s="29"/>
+      <c r="E83" s="27"/>
       <c r="F83" s="6" t="s">
         <v>44</v>
       </c>
@@ -7135,38 +7213,38 @@
       <c r="H83" s="6"/>
     </row>
     <row r="84" spans="1:8">
-      <c r="A84" s="53" t="s">
+      <c r="A84" s="44" t="s">
+        <v>208</v>
+      </c>
+      <c r="B84" s="6"/>
+      <c r="C84" s="23"/>
+      <c r="D84" s="37">
+        <v>246</v>
+      </c>
+      <c r="E84" s="27"/>
+      <c r="F84" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="B84" s="6"/>
-      <c r="C84" s="25"/>
-      <c r="D84" s="40">
-        <v>246</v>
-      </c>
-      <c r="E84" s="29"/>
-      <c r="F84" s="6" t="s">
+      <c r="G84" s="6" t="s">
         <v>210</v>
       </c>
-      <c r="G84" s="6" t="s">
-        <v>211</v>
-      </c>
       <c r="H84" s="6"/>
     </row>
     <row r="85" spans="1:8">
-      <c r="A85" s="54" t="s">
+      <c r="A85" s="45" t="s">
+        <v>215</v>
+      </c>
+      <c r="B85" s="6"/>
+      <c r="C85" s="23"/>
+      <c r="D85" s="37">
+        <v>247</v>
+      </c>
+      <c r="E85" s="27"/>
+      <c r="F85" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="B85" s="6"/>
-      <c r="C85" s="25"/>
-      <c r="D85" s="40">
-        <v>247</v>
-      </c>
-      <c r="E85" s="29"/>
-      <c r="F85" s="6" t="s">
+      <c r="G85" s="6" t="s">
         <v>217</v>
-      </c>
-      <c r="G85" s="6" t="s">
-        <v>218</v>
       </c>
       <c r="H85" s="6"/>
     </row>
@@ -7175,11 +7253,11 @@
         <v>27</v>
       </c>
       <c r="B86" s="6"/>
-      <c r="C86" s="25"/>
-      <c r="D86" s="40">
+      <c r="C86" s="23"/>
+      <c r="D86" s="37">
         <v>248</v>
       </c>
-      <c r="E86" s="29"/>
+      <c r="E86" s="27"/>
       <c r="F86" s="6" t="s">
         <v>45</v>
       </c>
@@ -7193,11 +7271,11 @@
         <v>182</v>
       </c>
       <c r="B87" s="6"/>
-      <c r="C87" s="25"/>
-      <c r="D87" s="40">
+      <c r="C87" s="23"/>
+      <c r="D87" s="37">
         <v>249</v>
       </c>
-      <c r="E87" s="29"/>
+      <c r="E87" s="27"/>
       <c r="F87" s="8" t="s">
         <v>183</v>
       </c>
@@ -7209,165 +7287,261 @@
       </c>
     </row>
     <row r="88" spans="1:8">
-      <c r="A88" s="53" t="s">
+      <c r="A88" s="44" t="s">
+        <v>205</v>
+      </c>
+      <c r="B88" s="6"/>
+      <c r="C88" s="23"/>
+      <c r="D88" s="37">
+        <v>250</v>
+      </c>
+      <c r="E88" s="27"/>
+      <c r="F88" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="B88" s="6"/>
-      <c r="C88" s="25"/>
-      <c r="D88" s="40">
+      <c r="G88" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="H88" s="6"/>
+    </row>
+    <row r="89" spans="1:8">
+      <c r="A89" s="45" t="s">
+        <v>222</v>
+      </c>
+      <c r="B89" s="6"/>
+      <c r="C89" s="23"/>
+      <c r="D89" s="37">
+        <v>251</v>
+      </c>
+      <c r="E89" s="27"/>
+      <c r="F89" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="G89" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="H89" s="8" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8">
+      <c r="A90" s="44" t="s">
+        <v>223</v>
+      </c>
+      <c r="B90" s="6"/>
+      <c r="C90" s="23"/>
+      <c r="D90" s="37">
+        <v>252</v>
+      </c>
+      <c r="E90" s="27"/>
+      <c r="F90" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="G90" s="6" t="s">
+        <v>228</v>
+      </c>
+      <c r="H90" s="8" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8">
+      <c r="A91" s="44" t="s">
+        <v>245</v>
+      </c>
+      <c r="B91" s="6"/>
+      <c r="C91" s="23"/>
+      <c r="D91" s="37">
+        <v>253</v>
+      </c>
+      <c r="E91" s="27"/>
+      <c r="F91" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="G91" s="6" t="s">
+        <v>246</v>
+      </c>
+      <c r="H91" s="8" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8">
+      <c r="A92" s="44" t="s">
+        <v>241</v>
+      </c>
+      <c r="B92" s="6"/>
+      <c r="C92" s="23"/>
+      <c r="D92" s="37">
+        <v>254</v>
+      </c>
+      <c r="E92" s="27"/>
+      <c r="F92" s="6" t="s">
+        <v>243</v>
+      </c>
+      <c r="G92" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="H92" s="8"/>
+    </row>
+    <row r="93" spans="1:8">
+      <c r="A93" s="44" t="s">
+        <v>242</v>
+      </c>
+      <c r="B93" s="6"/>
+      <c r="C93" s="23"/>
+      <c r="D93" s="37">
+        <v>255</v>
+      </c>
+      <c r="E93" s="27"/>
+      <c r="F93" s="6" t="s">
+        <v>244</v>
+      </c>
+      <c r="G93" s="6" t="s">
+        <v>252</v>
+      </c>
+      <c r="H93" s="8"/>
+    </row>
+    <row r="94" spans="1:8">
+      <c r="A94" s="44" t="s">
+        <v>253</v>
+      </c>
+      <c r="B94" s="6"/>
+      <c r="C94" s="23"/>
+      <c r="D94" s="37">
+        <v>256</v>
+      </c>
+      <c r="E94" s="27"/>
+      <c r="F94" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="G94" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="H94" s="8" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8">
+      <c r="A95" s="45" t="s">
+        <v>187</v>
+      </c>
+      <c r="B95" s="6"/>
+      <c r="C95" s="23"/>
+      <c r="D95" s="37">
+        <v>261</v>
+      </c>
+      <c r="E95" s="27"/>
+      <c r="F95" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="G95" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="H95" s="8"/>
+    </row>
+    <row r="96" spans="1:8">
+      <c r="A96" s="44" t="s">
+        <v>202</v>
+      </c>
+      <c r="B96" s="6"/>
+      <c r="C96" s="23"/>
+      <c r="D96" s="37">
+        <v>262</v>
+      </c>
+      <c r="E96" s="27"/>
+      <c r="F96" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="G96" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="H96" s="8"/>
+    </row>
+    <row r="97" spans="1:8">
+      <c r="A97" s="45" t="s">
+        <v>219</v>
+      </c>
+      <c r="B97" s="6"/>
+      <c r="C97" s="23"/>
+      <c r="D97" s="37">
+        <v>263</v>
+      </c>
+      <c r="E97" s="27"/>
+      <c r="F97" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="G97" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="H97" s="8" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="98" spans="1:8">
+      <c r="A98" s="44" t="s">
+        <v>224</v>
+      </c>
+      <c r="B98" s="6"/>
+      <c r="C98" s="23"/>
+      <c r="D98" s="37">
+        <v>264</v>
+      </c>
+      <c r="E98" s="27"/>
+      <c r="F98" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="G98" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="H98" s="8" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="99" spans="1:8">
+      <c r="A99" s="44" t="s">
+        <v>248</v>
+      </c>
+      <c r="B99" s="6"/>
+      <c r="C99" s="23"/>
+      <c r="D99" s="37">
+        <v>265</v>
+      </c>
+      <c r="E99" s="27"/>
+      <c r="F99" s="6" t="s">
+        <v>249</v>
+      </c>
+      <c r="G99" s="6" t="s">
         <v>250</v>
       </c>
-      <c r="E88" s="29"/>
-      <c r="F88" s="6" t="s">
-        <v>207</v>
-      </c>
-      <c r="G88" s="6" t="s">
-        <v>208</v>
-      </c>
-      <c r="H88" s="6"/>
-    </row>
-    <row r="89" spans="1:8">
-      <c r="A89" s="54" t="s">
-        <v>223</v>
-      </c>
-      <c r="B89" s="6"/>
-      <c r="C89" s="25"/>
-      <c r="D89" s="40">
-        <v>251</v>
-      </c>
-      <c r="E89" s="29"/>
-      <c r="F89" s="6" t="s">
-        <v>219</v>
-      </c>
-      <c r="G89" s="6" t="s">
-        <v>230</v>
-      </c>
-      <c r="H89" s="8" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="90" spans="1:8">
-      <c r="A90" s="53" t="s">
-        <v>224</v>
-      </c>
-      <c r="B90" s="6"/>
-      <c r="C90" s="25"/>
-      <c r="D90" s="40">
-        <v>252</v>
-      </c>
-      <c r="E90" s="29"/>
-      <c r="F90" s="6" t="s">
-        <v>228</v>
-      </c>
-      <c r="G90" s="6" t="s">
-        <v>229</v>
-      </c>
-      <c r="H90" s="8" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="91" spans="1:8">
-      <c r="A91" s="54" t="s">
-        <v>187</v>
-      </c>
-      <c r="B91" s="6"/>
-      <c r="C91" s="25"/>
-      <c r="D91" s="40">
-        <v>261</v>
-      </c>
-      <c r="E91" s="29"/>
-      <c r="F91" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="G91" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="H91" s="8"/>
-    </row>
-    <row r="92" spans="1:8">
-      <c r="A92" s="53" t="s">
-        <v>203</v>
-      </c>
-      <c r="B92" s="6"/>
-      <c r="C92" s="25"/>
-      <c r="D92" s="40">
-        <v>262</v>
-      </c>
-      <c r="E92" s="29"/>
-      <c r="F92" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="G92" s="6" t="s">
-        <v>205</v>
-      </c>
-      <c r="H92" s="8"/>
-    </row>
-    <row r="93" spans="1:8">
-      <c r="A93" s="54" t="s">
-        <v>220</v>
-      </c>
-      <c r="B93" s="6"/>
-      <c r="C93" s="25"/>
-      <c r="D93" s="40">
-        <v>263</v>
-      </c>
-      <c r="E93" s="29"/>
-      <c r="F93" s="6" t="s">
-        <v>221</v>
-      </c>
-      <c r="G93" s="6" t="s">
-        <v>222</v>
-      </c>
-      <c r="H93" s="8" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="94" spans="1:8">
-      <c r="A94" s="53" t="s">
-        <v>225</v>
-      </c>
-      <c r="B94" s="6"/>
-      <c r="C94" s="25"/>
-      <c r="D94" s="40">
-        <v>264</v>
-      </c>
-      <c r="E94" s="29"/>
-      <c r="F94" s="6" t="s">
-        <v>226</v>
-      </c>
-      <c r="G94" s="6" t="s">
-        <v>227</v>
-      </c>
-      <c r="H94" s="8" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="95" spans="1:8">
-      <c r="A95" s="1"/>
-      <c r="H95" s="4"/>
-    </row>
-    <row r="96" spans="1:8">
-      <c r="A96" s="1"/>
-      <c r="H96" s="4"/>
-    </row>
-    <row r="97" spans="1:8">
-      <c r="A97" s="1"/>
-      <c r="H97" s="4"/>
-    </row>
-    <row r="98" spans="1:8">
-      <c r="A98" s="1"/>
-    </row>
-    <row r="99" spans="1:8">
-      <c r="A99" s="1"/>
+      <c r="H99" s="8" t="s">
+        <v>232</v>
+      </c>
     </row>
     <row r="100" spans="1:8">
       <c r="A100" s="1"/>
+      <c r="H100" s="4"/>
     </row>
     <row r="101" spans="1:8">
       <c r="A101" s="1"/>
+      <c r="H101" s="4"/>
     </row>
     <row r="102" spans="1:8">
       <c r="A102" s="1"/>
+      <c r="H102" s="4"/>
+    </row>
+    <row r="103" spans="1:8">
+      <c r="A103" s="1"/>
+    </row>
+    <row r="104" spans="1:8">
+      <c r="A104" s="1"/>
+    </row>
+    <row r="105" spans="1:8">
+      <c r="A105" s="1"/>
+    </row>
+    <row r="106" spans="1:8">
+      <c r="A106" s="1"/>
+    </row>
+    <row r="107" spans="1:8">
+      <c r="A107" s="1"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A7:C17">

</xml_diff>